<commit_message>
Attempt at better EKF flow
</commit_message>
<xml_diff>
--- a/OD Project Code Architecture.xlsx
+++ b/OD Project Code Architecture.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isaac\Documents\Spring_2026\Methods of Orbital Determination\Methods_OD_Final_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954DF80A-4715-4D06-A3D4-253B7BC7795C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B83FF0A-5D23-4DA7-BCE6-FA32A4B76432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="10090" windowHeight="11370" xr2:uid="{27519F2F-6E3C-4B5D-A672-E70B8865A5DC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{27519F2F-6E3C-4B5D-A672-E70B8865A5DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
   <si>
     <t>Initial Conditions, Settings, Environment</t>
   </si>
@@ -53,7 +53,118 @@
     <t>Plotting</t>
   </si>
   <si>
-    <t>Filter Settings (Which Date Sets/Types)</t>
+    <t>Load EOP Data</t>
+  </si>
+  <si>
+    <t>Load Reference Data</t>
+  </si>
+  <si>
+    <t>Load mex/MatlabFunctions</t>
+  </si>
+  <si>
+    <t>Compute Any Remaining Initial Conditions</t>
+  </si>
+  <si>
+    <t>Filters</t>
+  </si>
+  <si>
+    <t>Batch</t>
+  </si>
+  <si>
+    <t>EKF</t>
+  </si>
+  <si>
+    <t>UKF?</t>
+  </si>
+  <si>
+    <t>Measurement Model &amp; Tools</t>
+  </si>
+  <si>
+    <t>Dynamics Model &amp; Tools</t>
+  </si>
+  <si>
+    <t>Visualization Tools</t>
+  </si>
+  <si>
+    <t>Misc. Tools</t>
+  </si>
+  <si>
+    <t>Settings (Filter Data Sets/Types, Dynamics Models, etc.)</t>
+  </si>
+  <si>
+    <t>Settings/Data Logger</t>
+  </si>
+  <si>
+    <t>Settings/Data Loader</t>
+  </si>
+  <si>
+    <t>Gravity (Simple + J2)</t>
+  </si>
+  <si>
+    <t>LuniSolar Pertubations</t>
+  </si>
+  <si>
+    <t>Solar Radiation Pressure</t>
+  </si>
+  <si>
+    <t>Drag</t>
+  </si>
+  <si>
+    <t>Spherical Harmonics (20x20 EGM96)</t>
+  </si>
+  <si>
+    <t>ECEF_to_ECI</t>
+  </si>
+  <si>
+    <t>ECI_to_ECEF</t>
+  </si>
+  <si>
+    <t>Sun, Moon Positions</t>
+  </si>
+  <si>
+    <t>Constants</t>
+  </si>
+  <si>
+    <t>jah_sat_1_ode</t>
+  </si>
+  <si>
+    <t>Total Acceraration Function</t>
+  </si>
+  <si>
+    <t>A Matrix Computation Function</t>
+  </si>
+  <si>
+    <t>Range &amp; Range_Rate Modeler</t>
+  </si>
+  <si>
+    <t>Measurement Computation</t>
+  </si>
+  <si>
+    <t>H Matrix Computation</t>
+  </si>
+  <si>
+    <t>Compute Observation (with ECI/ECEF Conversion)</t>
+  </si>
+  <si>
+    <t>Plot Pre/Post-fit Residuals</t>
+  </si>
+  <si>
+    <t>Total Orbit</t>
+  </si>
+  <si>
+    <t>RIC (Thundering Herd)</t>
+  </si>
+  <si>
+    <t>Plot Acceleration Vectors</t>
+  </si>
+  <si>
+    <t>3D Animation</t>
+  </si>
+  <si>
+    <t>Output: Struct with values</t>
+  </si>
+  <si>
+    <t>Output: Struct with booleans for settings</t>
   </si>
 </sst>
 </file>
@@ -70,6 +181,7 @@
     </font>
     <font>
       <b/>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -434,37 +546,181 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{418E5AFC-DC86-4343-A89C-4F3B4C2D0513}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="47.08984375" customWidth="1"/>
+    <col min="3" max="6" width="35.90625" customWidth="1"/>
+    <col min="7" max="8" width="26.36328125" customWidth="1"/>
+    <col min="9" max="10" width="26.1796875" customWidth="1"/>
+    <col min="11" max="11" width="21.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>